<commit_message>
MenuFiller works, needs integration into app.py
</commit_message>
<xml_diff>
--- a/refactor/output.xlsx
+++ b/refactor/output.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4020" yWindow="4530" windowWidth="19080" windowHeight="15345" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="menu_template" sheetId="1" state="visible" r:id="rId1"/>
@@ -1779,7 +1779,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:IV13"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="14.42578125" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="18" customWidth="1" style="1" min="1" max="2"/>
     <col width="19.42578125" customWidth="1" style="1" min="3" max="3"/>
@@ -1789,10 +1789,8 @@
   </cols>
   <sheetData>
     <row r="1" ht="50.1" customFormat="1" customHeight="1" s="3" thickBot="1">
-      <c r="A1" s="39" t="inlineStr">
-        <is>
-          <t>29/08/2022</t>
-        </is>
+      <c r="A1" s="39" t="n">
+        <v>46027</v>
       </c>
       <c r="B1" s="5" t="n"/>
       <c r="C1" s="50" t="n"/>
@@ -2211,36 +2209,84 @@
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
-          <t>Appetizer</t>
+          <t>Soup &amp; Appetizer</t>
         </is>
       </c>
       <c r="E4" s="15" t="inlineStr">
         <is>
-          <t>Entrée</t>
+          <t>Soupe &amp; Entrée</t>
         </is>
       </c>
       <c r="F4" s="16" t="inlineStr">
         <is>
-          <t>soupe au poulet   et nouilles</t>
+          <t>Soupe rustique aux légumineuses  + Trempette chaude aux poireaux et  cheddar</t>
         </is>
       </c>
       <c r="G4" s="17" t="inlineStr">
         <is>
-          <t>Chicken soup and noodles</t>
-        </is>
-      </c>
-      <c r="H4" s="16" t="n"/>
-      <c r="I4" s="17" t="n"/>
-      <c r="J4" s="16" t="n"/>
-      <c r="K4" s="17" t="n"/>
-      <c r="L4" s="16" t="n"/>
-      <c r="M4" s="17" t="n"/>
-      <c r="N4" s="16" t="n"/>
-      <c r="O4" s="17" t="n"/>
-      <c r="P4" s="16" t="n"/>
-      <c r="Q4" s="17" t="n"/>
-      <c r="R4" s="16" t="n"/>
-      <c r="S4" s="17" t="n"/>
+          <t>translate this : Soupe rustique aux légumineuses  &lt;-- + translate this : Trempette chaude aux poireaux et  cheddar &lt;--</t>
+        </is>
+      </c>
+      <c r="H4" s="16" t="inlineStr">
+        <is>
+          <t>Potage Freneuse au miel (navets) + Salade de concombres et yogourt (OF)</t>
+        </is>
+      </c>
+      <c r="I4" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Potage Freneuse au miel (navets) &lt;-- + translate this : Salade de concombres et yogourt (OF) &lt;--</t>
+        </is>
+      </c>
+      <c r="J4" s="16" t="inlineStr">
+        <is>
+          <t>Chaudrée de maïs et jambon  + Dumpling au poulet et vinaigrette au sésame</t>
+        </is>
+      </c>
+      <c r="K4" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Chaudrée de maïs et jambon  &lt;-- + translate this : Dumpling au poulet et vinaigrette au sésame &lt;--</t>
+        </is>
+      </c>
+      <c r="L4" s="16" t="inlineStr">
+        <is>
+          <t>Velouté de courge butternut  + Fondue parmesan et roquette</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Velouté de courge butternut  &lt;-- + translate this : Fondue parmesan et roquette &lt;--</t>
+        </is>
+      </c>
+      <c r="N4" s="16" t="inlineStr">
+        <is>
+          <t>Crème de brocoli au basilic + Salade de betteraves, au chèvre (QC)</t>
+        </is>
+      </c>
+      <c r="O4" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Crème de brocoli au basilic &lt;-- + translate this : Salade de betteraves, au chèvre (QC) &lt;--</t>
+        </is>
+      </c>
+      <c r="P4" s="16" t="inlineStr">
+        <is>
+          <t>Soupe minestrone + Salade aux épinards, mandarines et parmesan</t>
+        </is>
+      </c>
+      <c r="Q4" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Soupe minestrone &lt;-- + translate this : Salade aux épinards, mandarines et parmesan &lt;--</t>
+        </is>
+      </c>
+      <c r="R4" s="16" t="inlineStr">
+        <is>
+          <t>Crème de  poireaux  + Salade de pommes de terre à l’estragon</t>
+        </is>
+      </c>
+      <c r="S4" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Crème de  poireaux  &lt;-- + translate this : Salade de pommes de terre à l’estragon &lt;--</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="65.09999999999999" customHeight="1" s="1">
       <c r="A5" s="18" t="n"/>
@@ -2248,36 +2294,84 @@
       <c r="C5" s="20" t="n"/>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>Appetizer</t>
+          <t>Main course</t>
         </is>
       </c>
       <c r="E5" s="15" t="inlineStr">
         <is>
-          <t>Entrée</t>
+          <t>Plat principal</t>
         </is>
       </c>
       <c r="F5" s="16" t="inlineStr">
         <is>
-          <t>salade de bettraves   et  fromage feta</t>
+          <t>Hot Chicken (C)</t>
         </is>
       </c>
       <c r="G5" s="17" t="inlineStr">
         <is>
-          <t>Beet salad and feta cheese</t>
-        </is>
-      </c>
-      <c r="H5" s="16" t="n"/>
-      <c r="I5" s="17" t="n"/>
-      <c r="J5" s="16" t="n"/>
-      <c r="K5" s="17" t="n"/>
-      <c r="L5" s="16" t="n"/>
-      <c r="M5" s="17" t="n"/>
-      <c r="N5" s="16" t="n"/>
-      <c r="O5" s="17" t="n"/>
-      <c r="P5" s="16" t="n"/>
-      <c r="Q5" s="17" t="n"/>
-      <c r="R5" s="16" t="n"/>
-      <c r="S5" s="17" t="n"/>
+          <t>translate this : Hot Chicken (C) &lt;--</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">joue de porc au jus </t>
+        </is>
+      </c>
+      <c r="I5" s="17" t="inlineStr">
+        <is>
+          <t>translate this : joue de porc au jus  &lt;--</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Hamburger steak (C) </t>
+        </is>
+      </c>
+      <c r="K5" s="17" t="inlineStr">
+        <is>
+          <t>translate this :  Hamburger steak (C)  &lt;--</t>
+        </is>
+      </c>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Penne a la gigi </t>
+        </is>
+      </c>
+      <c r="M5" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Penne a la gigi  &lt;--</t>
+        </is>
+      </c>
+      <c r="N5" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">longe de porc aux pommes </t>
+        </is>
+      </c>
+      <c r="O5" s="17" t="inlineStr">
+        <is>
+          <t>translate this : longe de porc aux pommes  &lt;--</t>
+        </is>
+      </c>
+      <c r="P5" s="16" t="inlineStr">
+        <is>
+          <t>Rôti de palette balsamique et oignons</t>
+        </is>
+      </c>
+      <c r="Q5" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Rôti de palette balsamique et oignons &lt;--</t>
+        </is>
+      </c>
+      <c r="R5" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Brunch </t>
+        </is>
+      </c>
+      <c r="S5" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Brunch  &lt;--</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="65.09999999999999" customHeight="1" s="1">
       <c r="A6" s="18" t="n"/>
@@ -2295,26 +2389,74 @@
       </c>
       <c r="F6" s="16" t="inlineStr">
         <is>
-          <t>wrap a la dinde au bacon , laitue et tomate</t>
+          <t>Linguine Alfredo aux fruits de mer</t>
         </is>
       </c>
       <c r="G6" s="17" t="inlineStr">
         <is>
-          <t>wrap has turkey in bacon, lettuce and tomato</t>
-        </is>
-      </c>
-      <c r="H6" s="16" t="n"/>
-      <c r="I6" s="17" t="n"/>
-      <c r="J6" s="16" t="n"/>
-      <c r="K6" s="17" t="n"/>
-      <c r="L6" s="16" t="n"/>
-      <c r="M6" s="17" t="n"/>
-      <c r="N6" s="16" t="n"/>
-      <c r="O6" s="17" t="n"/>
-      <c r="P6" s="16" t="n"/>
-      <c r="Q6" s="17" t="n"/>
-      <c r="R6" s="16" t="n"/>
-      <c r="S6" s="17" t="n"/>
+          <t>translate this : Linguine Alfredo aux fruits de mer &lt;--</t>
+        </is>
+      </c>
+      <c r="H6" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Braisé de veau à la  hongroise </t>
+        </is>
+      </c>
+      <c r="I6" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Braisé de veau à la  hongroise  &lt;--</t>
+        </is>
+      </c>
+      <c r="J6" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Coquille aux fruits de mer gratinée (C) </t>
+        </is>
+      </c>
+      <c r="K6" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Coquille aux fruits de mer gratinée (C)  &lt;--</t>
+        </is>
+      </c>
+      <c r="L6" s="16" t="inlineStr">
+        <is>
+          <t>Haut de cuisse de poulet grillés à la sauce teriyaki</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Haut de cuisse de poulet grillés à la sauce teriyaki &lt;--</t>
+        </is>
+      </c>
+      <c r="N6" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">salade de poulet cesar </t>
+        </is>
+      </c>
+      <c r="O6" s="17" t="inlineStr">
+        <is>
+          <t>translate this : salade de poulet cesar  &lt;--</t>
+        </is>
+      </c>
+      <c r="P6" s="16" t="inlineStr">
+        <is>
+          <t>Filets de colin au basilic</t>
+        </is>
+      </c>
+      <c r="Q6" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Filets de colin au basilic &lt;--</t>
+        </is>
+      </c>
+      <c r="R6" s="16" t="inlineStr">
+        <is>
+          <t>Mijoté de bœuf aux navets et pommes de terre</t>
+        </is>
+      </c>
+      <c r="S6" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Mijoté de bœuf aux navets et pommes de terre &lt;--</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="65.09999999999999" customHeight="1" s="1">
       <c r="A7" s="18" t="n"/>
@@ -2332,26 +2474,74 @@
       </c>
       <c r="F7" s="16" t="inlineStr">
         <is>
-          <t>filet de tilapia sauce  salsa verde</t>
+          <t>Salade grecque (I)</t>
         </is>
       </c>
       <c r="G7" s="17" t="inlineStr">
         <is>
-          <t>Tilapia Sauce Filet Green Sauce</t>
-        </is>
-      </c>
-      <c r="H7" s="16" t="n"/>
-      <c r="I7" s="17" t="n"/>
-      <c r="J7" s="16" t="n"/>
-      <c r="K7" s="17" t="n"/>
-      <c r="L7" s="16" t="n"/>
-      <c r="M7" s="17" t="n"/>
-      <c r="N7" s="16" t="n"/>
-      <c r="O7" s="17" t="n"/>
-      <c r="P7" s="16" t="n"/>
-      <c r="Q7" s="17" t="n"/>
-      <c r="R7" s="16" t="n"/>
-      <c r="S7" s="17" t="n"/>
+          <t>translate this : Salade grecque (I) &lt;--</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sauté de poulet mangue coco (I) </t>
+        </is>
+      </c>
+      <c r="I7" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Sauté de poulet mangue coco (I)  &lt;--</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>Orgetto aux champignons (I)</t>
+        </is>
+      </c>
+      <c r="K7" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Orgetto aux champignons (I) &lt;--</t>
+        </is>
+      </c>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Crevettes à la créole (I) </t>
+        </is>
+      </c>
+      <c r="M7" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Crevettes à la créole (I)  &lt;--</t>
+        </is>
+      </c>
+      <c r="N7" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pâtes au saumon fumé(I) </t>
+        </is>
+      </c>
+      <c r="O7" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Pâtes au saumon fumé(I)  &lt;--</t>
+        </is>
+      </c>
+      <c r="P7" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dinde miel et ail (I) </t>
+        </is>
+      </c>
+      <c r="Q7" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Dinde miel et ail (I)  &lt;--</t>
+        </is>
+      </c>
+      <c r="R7" s="16" t="inlineStr">
+        <is>
+          <t>Filet de sole salsa de tomates (I)</t>
+        </is>
+      </c>
+      <c r="S7" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Filet de sole salsa de tomates (I) &lt;--</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="65.09999999999999" customHeight="1" s="1">
       <c r="A8" s="18" t="n"/>
@@ -2369,26 +2559,74 @@
       </c>
       <c r="F8" s="16" t="inlineStr">
         <is>
-          <t>tarte au sucre</t>
+          <t xml:space="preserve">Beigne glacé à l'érable </t>
         </is>
       </c>
       <c r="G8" s="17" t="inlineStr">
         <is>
-          <t>sugar pie</t>
-        </is>
-      </c>
-      <c r="H8" s="16" t="n"/>
-      <c r="I8" s="17" t="n"/>
-      <c r="J8" s="16" t="n"/>
-      <c r="K8" s="17" t="n"/>
-      <c r="L8" s="16" t="n"/>
-      <c r="M8" s="17" t="n"/>
-      <c r="N8" s="16" t="n"/>
-      <c r="O8" s="17" t="n"/>
-      <c r="P8" s="16" t="n"/>
-      <c r="Q8" s="17" t="n"/>
-      <c r="R8" s="16" t="n"/>
-      <c r="S8" s="17" t="n"/>
+          <t>translate this : Beigne glacé à l'érable  &lt;--</t>
+        </is>
+      </c>
+      <c r="H8" s="16" t="inlineStr">
+        <is>
+          <t>Assortis</t>
+        </is>
+      </c>
+      <c r="I8" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Assortis &lt;--</t>
+        </is>
+      </c>
+      <c r="J8" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cannoli a la creme </t>
+        </is>
+      </c>
+      <c r="K8" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Cannoli a la creme  &lt;--</t>
+        </is>
+      </c>
+      <c r="L8" s="16" t="inlineStr">
+        <is>
+          <t>Profiterole au chocolat</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Profiterole au chocolat &lt;--</t>
+        </is>
+      </c>
+      <c r="N8" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tarte citron </t>
+        </is>
+      </c>
+      <c r="O8" s="17" t="inlineStr">
+        <is>
+          <t>translate this : tarte citron  &lt;--</t>
+        </is>
+      </c>
+      <c r="P8" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assortis </t>
+        </is>
+      </c>
+      <c r="Q8" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Assortis  &lt;--</t>
+        </is>
+      </c>
+      <c r="R8" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gateaux vanille et fraise </t>
+        </is>
+      </c>
+      <c r="S8" s="17" t="inlineStr">
+        <is>
+          <t>translate this : gateaux vanille et fraise  &lt;--</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="65.09999999999999" customHeight="1" s="1">
       <c r="A9" s="21" t="inlineStr">
@@ -2408,36 +2646,84 @@
       </c>
       <c r="D9" s="23" t="inlineStr">
         <is>
-          <t>Appetizer</t>
+          <t>Soup &amp; Appetizer</t>
         </is>
       </c>
       <c r="E9" s="24" t="inlineStr">
         <is>
-          <t>Entrée</t>
+          <t>Soupe &amp; Entrée</t>
         </is>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>creme de celeri rave au miel</t>
+          <t>Potage Freneuse au miel (navets) + Salade de concombres et yogourt (OF)</t>
         </is>
       </c>
       <c r="G9" s="17" t="inlineStr">
         <is>
-          <t>Cream of Celeri Rave with honey</t>
-        </is>
-      </c>
-      <c r="H9" s="25" t="n"/>
-      <c r="I9" s="17" t="n"/>
-      <c r="J9" s="25" t="n"/>
-      <c r="K9" s="17" t="n"/>
-      <c r="L9" s="25" t="n"/>
-      <c r="M9" s="26" t="n"/>
-      <c r="N9" s="25" t="n"/>
-      <c r="O9" s="17" t="n"/>
-      <c r="P9" s="25" t="n"/>
-      <c r="Q9" s="17" t="n"/>
-      <c r="R9" s="25" t="n"/>
-      <c r="S9" s="17" t="n"/>
+          <t>translate this : Potage Freneuse au miel (navets) &lt;-- + translate this : Salade de concombres et yogourt (OF) &lt;--</t>
+        </is>
+      </c>
+      <c r="H9" s="25" t="inlineStr">
+        <is>
+          <t>Chaudrée de maïs et jambon  + Dumpling au poulet et vinaigrette au sésame</t>
+        </is>
+      </c>
+      <c r="I9" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Chaudrée de maïs et jambon  &lt;-- + translate this : Dumpling au poulet et vinaigrette au sésame &lt;--</t>
+        </is>
+      </c>
+      <c r="J9" s="25" t="inlineStr">
+        <is>
+          <t>Velouté de courge butternut  + Fondue parmesan et roquette</t>
+        </is>
+      </c>
+      <c r="K9" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Velouté de courge butternut  &lt;-- + translate this : Fondue parmesan et roquette &lt;--</t>
+        </is>
+      </c>
+      <c r="L9" s="25" t="inlineStr">
+        <is>
+          <t>Crème de brocoli au basilic + Salade de betteraves, au chèvre (QC)</t>
+        </is>
+      </c>
+      <c r="M9" s="26" t="inlineStr">
+        <is>
+          <t>translate this : Crème de brocoli au basilic &lt;-- + translate this : Salade de betteraves, au chèvre (QC) &lt;--</t>
+        </is>
+      </c>
+      <c r="N9" s="25" t="inlineStr">
+        <is>
+          <t>Soupe minestrone + Salade aux épinards, mandarines et parmesan</t>
+        </is>
+      </c>
+      <c r="O9" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Soupe minestrone &lt;-- + translate this : Salade aux épinards, mandarines et parmesan &lt;--</t>
+        </is>
+      </c>
+      <c r="P9" s="25" t="inlineStr">
+        <is>
+          <t>Crème de  poireaux  + Salade de pommes de terre à l’estragon</t>
+        </is>
+      </c>
+      <c r="Q9" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Crème de  poireaux  &lt;-- + translate this : Salade de pommes de terre à l’estragon &lt;--</t>
+        </is>
+      </c>
+      <c r="R9" s="25" t="inlineStr">
+        <is>
+          <t>Velouté de patate douce au lait de coco et gingembre (QC) + Rillette de saumonfumé et basilic</t>
+        </is>
+      </c>
+      <c r="S9" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Velouté de patate douce au lait de coco et gingembre (QC) &lt;-- + translate this : Rillette de saumonfumé et basilic &lt;--</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="65.09999999999999" customHeight="1" s="1">
       <c r="A10" s="27" t="n"/>
@@ -2445,36 +2731,84 @@
       <c r="C10" s="29" t="n"/>
       <c r="D10" s="23" t="inlineStr">
         <is>
-          <t>Appetizer</t>
+          <t>Main course</t>
         </is>
       </c>
       <c r="E10" s="24" t="inlineStr">
         <is>
-          <t>Entrée</t>
+          <t>Plat principal</t>
         </is>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>salade de bettraves   et  fromage feta</t>
+          <t>Hot Chicken (C)</t>
         </is>
       </c>
       <c r="G10" s="17" t="inlineStr">
         <is>
-          <t>Beet salad and feta cheese</t>
-        </is>
-      </c>
-      <c r="H10" s="25" t="n"/>
-      <c r="I10" s="17" t="n"/>
-      <c r="J10" s="25" t="n"/>
-      <c r="K10" s="17" t="n"/>
-      <c r="L10" s="25" t="n"/>
-      <c r="M10" s="17" t="n"/>
-      <c r="N10" s="25" t="n"/>
-      <c r="O10" s="17" t="n"/>
-      <c r="P10" s="25" t="n"/>
-      <c r="Q10" s="17" t="n"/>
-      <c r="R10" s="25" t="n"/>
-      <c r="S10" s="17" t="n"/>
+          <t>translate this : Hot Chicken (C) &lt;--</t>
+        </is>
+      </c>
+      <c r="H10" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">joue de porc au jus </t>
+        </is>
+      </c>
+      <c r="I10" s="17" t="inlineStr">
+        <is>
+          <t>translate this : joue de porc au jus  &lt;--</t>
+        </is>
+      </c>
+      <c r="J10" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Hamburger steak (C) </t>
+        </is>
+      </c>
+      <c r="K10" s="17" t="inlineStr">
+        <is>
+          <t>translate this :  Hamburger steak (C)  &lt;--</t>
+        </is>
+      </c>
+      <c r="L10" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Penne a la gigi </t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Penne a la gigi  &lt;--</t>
+        </is>
+      </c>
+      <c r="N10" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">longe de porc aux pommes </t>
+        </is>
+      </c>
+      <c r="O10" s="17" t="inlineStr">
+        <is>
+          <t>translate this : longe de porc aux pommes  &lt;--</t>
+        </is>
+      </c>
+      <c r="P10" s="25" t="inlineStr">
+        <is>
+          <t>Rôti de palette balsamique et oignons</t>
+        </is>
+      </c>
+      <c r="Q10" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Rôti de palette balsamique et oignons &lt;--</t>
+        </is>
+      </c>
+      <c r="R10" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Brunch </t>
+        </is>
+      </c>
+      <c r="S10" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Brunch  &lt;--</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="65.09999999999999" customHeight="1" s="1">
       <c r="A11" s="30" t="n"/>
@@ -2492,26 +2826,74 @@
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
-          <t>mijoté de veau a la lime et au paprika fumé</t>
+          <t>Linguine Alfredo aux fruits de mer</t>
         </is>
       </c>
       <c r="G11" s="17" t="inlineStr">
         <is>
-          <t>veal simmer with lime and smoked paprika</t>
-        </is>
-      </c>
-      <c r="H11" s="25" t="n"/>
-      <c r="I11" s="17" t="n"/>
-      <c r="J11" s="25" t="n"/>
-      <c r="K11" s="17" t="n"/>
-      <c r="L11" s="25" t="n"/>
-      <c r="M11" s="26" t="n"/>
-      <c r="N11" s="25" t="n"/>
-      <c r="O11" s="17" t="n"/>
-      <c r="P11" s="25" t="n"/>
-      <c r="Q11" s="17" t="n"/>
-      <c r="R11" s="25" t="n"/>
-      <c r="S11" s="17" t="n"/>
+          <t>translate this : Linguine Alfredo aux fruits de mer &lt;--</t>
+        </is>
+      </c>
+      <c r="H11" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Braisé de veau à la  hongroise </t>
+        </is>
+      </c>
+      <c r="I11" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Braisé de veau à la  hongroise  &lt;--</t>
+        </is>
+      </c>
+      <c r="J11" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Coquille aux fruits de mer gratinée (C) </t>
+        </is>
+      </c>
+      <c r="K11" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Coquille aux fruits de mer gratinée (C)  &lt;--</t>
+        </is>
+      </c>
+      <c r="L11" s="25" t="inlineStr">
+        <is>
+          <t>Haut de cuisse de poulet grillés à la sauce teriyaki</t>
+        </is>
+      </c>
+      <c r="M11" s="26" t="inlineStr">
+        <is>
+          <t>translate this : Haut de cuisse de poulet grillés à la sauce teriyaki &lt;--</t>
+        </is>
+      </c>
+      <c r="N11" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">salade de poulet cesar </t>
+        </is>
+      </c>
+      <c r="O11" s="17" t="inlineStr">
+        <is>
+          <t>translate this : salade de poulet cesar  &lt;--</t>
+        </is>
+      </c>
+      <c r="P11" s="25" t="inlineStr">
+        <is>
+          <t>Filets de colin au basilic</t>
+        </is>
+      </c>
+      <c r="Q11" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Filets de colin au basilic &lt;--</t>
+        </is>
+      </c>
+      <c r="R11" s="25" t="inlineStr">
+        <is>
+          <t>Mijoté de bœuf aux navets et pommes de terre</t>
+        </is>
+      </c>
+      <c r="S11" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Mijoté de bœuf aux navets et pommes de terre &lt;--</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="65.09999999999999" customHeight="1" s="1">
       <c r="A12" s="30" t="n"/>
@@ -2529,26 +2911,74 @@
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>lasagne a la viande gratinée</t>
+          <t>Salade grecque (I)</t>
         </is>
       </c>
       <c r="G12" s="17" t="inlineStr">
         <is>
-          <t>gratin meat lasagna</t>
-        </is>
-      </c>
-      <c r="H12" s="25" t="n"/>
-      <c r="I12" s="17" t="n"/>
-      <c r="J12" s="25" t="n"/>
-      <c r="K12" s="17" t="n"/>
-      <c r="L12" s="25" t="n"/>
-      <c r="M12" s="26" t="n"/>
-      <c r="N12" s="25" t="n"/>
-      <c r="O12" s="17" t="n"/>
-      <c r="P12" s="25" t="n"/>
-      <c r="Q12" s="17" t="n"/>
-      <c r="R12" s="25" t="n"/>
-      <c r="S12" s="17" t="n"/>
+          <t>translate this : Salade grecque (I) &lt;--</t>
+        </is>
+      </c>
+      <c r="H12" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sauté de poulet mangue coco (I) </t>
+        </is>
+      </c>
+      <c r="I12" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Sauté de poulet mangue coco (I)  &lt;--</t>
+        </is>
+      </c>
+      <c r="J12" s="25" t="inlineStr">
+        <is>
+          <t>Orgetto aux champignons (I)</t>
+        </is>
+      </c>
+      <c r="K12" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Orgetto aux champignons (I) &lt;--</t>
+        </is>
+      </c>
+      <c r="L12" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Crevettes à la créole (I) </t>
+        </is>
+      </c>
+      <c r="M12" s="26" t="inlineStr">
+        <is>
+          <t>translate this : Crevettes à la créole (I)  &lt;--</t>
+        </is>
+      </c>
+      <c r="N12" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pâtes au saumon fumé(I) </t>
+        </is>
+      </c>
+      <c r="O12" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Pâtes au saumon fumé(I)  &lt;--</t>
+        </is>
+      </c>
+      <c r="P12" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dinde miel et ail (I) </t>
+        </is>
+      </c>
+      <c r="Q12" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Dinde miel et ail (I)  &lt;--</t>
+        </is>
+      </c>
+      <c r="R12" s="25" t="inlineStr">
+        <is>
+          <t>Filet de sole salsa de tomates (I)</t>
+        </is>
+      </c>
+      <c r="S12" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Filet de sole salsa de tomates (I) &lt;--</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="65.09999999999999" customHeight="1" s="1" thickBot="1">
       <c r="A13" s="32" t="n"/>
@@ -2566,26 +2996,74 @@
       </c>
       <c r="F13" s="37" t="inlineStr">
         <is>
-          <t>tarte au sucre</t>
+          <t>Assortis</t>
         </is>
       </c>
       <c r="G13" s="17" t="inlineStr">
         <is>
-          <t>sugar pie</t>
-        </is>
-      </c>
-      <c r="H13" s="37" t="n"/>
-      <c r="I13" s="38" t="n"/>
-      <c r="J13" s="37" t="n"/>
-      <c r="K13" s="17" t="n"/>
-      <c r="L13" s="37" t="n"/>
-      <c r="M13" s="17" t="n"/>
-      <c r="N13" s="37" t="n"/>
-      <c r="O13" s="17" t="n"/>
-      <c r="P13" s="37" t="n"/>
-      <c r="Q13" s="17" t="n"/>
-      <c r="R13" s="37" t="n"/>
-      <c r="S13" s="17" t="n"/>
+          <t>translate this : Assortis &lt;--</t>
+        </is>
+      </c>
+      <c r="H13" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cannoli a la creme </t>
+        </is>
+      </c>
+      <c r="I13" s="38" t="inlineStr">
+        <is>
+          <t>translate this : Cannoli a la creme  &lt;--</t>
+        </is>
+      </c>
+      <c r="J13" s="37" t="inlineStr">
+        <is>
+          <t>Profiterole au chocolat</t>
+        </is>
+      </c>
+      <c r="K13" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Profiterole au chocolat &lt;--</t>
+        </is>
+      </c>
+      <c r="L13" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tarte citron </t>
+        </is>
+      </c>
+      <c r="M13" s="17" t="inlineStr">
+        <is>
+          <t>translate this : tarte citron  &lt;--</t>
+        </is>
+      </c>
+      <c r="N13" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assortis </t>
+        </is>
+      </c>
+      <c r="O13" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Assortis  &lt;--</t>
+        </is>
+      </c>
+      <c r="P13" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gateaux vanille et fraise </t>
+        </is>
+      </c>
+      <c r="Q13" s="17" t="inlineStr">
+        <is>
+          <t>translate this : gateaux vanille et fraise  &lt;--</t>
+        </is>
+      </c>
+      <c r="R13" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Brownie moelleux chocolat </t>
+        </is>
+      </c>
+      <c r="S13" s="17" t="inlineStr">
+        <is>
+          <t>translate this : Brownie moelleux chocolat  &lt;--</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>